<commit_message>
Admin pannel Auto logout in 30 mint done
</commit_message>
<xml_diff>
--- a/server/uploads/reports/WeeklyTaskReport_2026-07-12_to_2026-07-18.xlsx
+++ b/server/uploads/reports/WeeklyTaskReport_2026-07-12_to_2026-07-18.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="15">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="34" uniqueCount="21">
   <si>
     <t>Weekly Task Report (12/7/2026 to 18/7/2026)</t>
   </si>
@@ -50,6 +50,24 @@
   </si>
   <si>
     <t>Mohammad Mazhar</t>
+  </si>
+  <si>
+    <t>Priti Bandewar</t>
+  </si>
+  <si>
+    <t>1.00</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ai doctor voice </t>
+  </si>
+  <si>
+    <t>0.83</t>
+  </si>
+  <si>
+    <t>testing by priti</t>
+  </si>
+  <si>
+    <t>0.17</t>
   </si>
   <si>
     <t>PALAK RAIKWAR</t>
@@ -454,7 +472,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F12"/>
+  <dimension ref="A1:F16"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="6" width="45" customWidth="1"/>
@@ -587,10 +605,10 @@
         <v>0</v>
       </c>
       <c r="E10" s="3">
-        <v>200</v>
+        <v>60</v>
       </c>
       <c r="F10" s="3" t="s">
-        <v>9</v>
+        <v>14</v>
       </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.25">
@@ -598,7 +616,7 @@
         <v>10</v>
       </c>
       <c r="B11" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="C11">
         <v>0</v>
@@ -607,13 +625,74 @@
         <v>0</v>
       </c>
       <c r="E11">
+        <v>50</v>
+      </c>
+      <c r="F11" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>10</v>
+      </c>
+      <c r="B12" t="s">
+        <v>17</v>
+      </c>
+      <c r="C12">
+        <v>0</v>
+      </c>
+      <c r="D12">
+        <v>0</v>
+      </c>
+      <c r="E12">
+        <v>10</v>
+      </c>
+      <c r="F12" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.25"/>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A14" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="B14" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="C14" s="3">
+        <v>0</v>
+      </c>
+      <c r="D14" s="3">
+        <v>0</v>
+      </c>
+      <c r="E14" s="3">
         <v>200</v>
       </c>
-      <c r="F11" t="s">
+      <c r="F14" s="3" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.25"/>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>10</v>
+      </c>
+      <c r="B15" t="s">
+        <v>20</v>
+      </c>
+      <c r="C15">
+        <v>0</v>
+      </c>
+      <c r="D15">
+        <v>0</v>
+      </c>
+      <c r="E15">
+        <v>200</v>
+      </c>
+      <c r="F15" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" x14ac:dyDescent="0.25"/>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:F1"/>

</xml_diff>